<commit_message>
add remessa 016 fertilidade
</commit_message>
<xml_diff>
--- a/pedidos/PAV2026002S.xlsx
+++ b/pedidos/PAV2026002S.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/pedidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{3EE82390-A8D5-4DA9-852E-5EE8943864DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEC5AF7B-1DA0-4ECB-A52C-298F91ADB04F}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{3EE82390-A8D5-4DA9-852E-5EE8943864DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C046AA1-C3DB-408B-964A-AE6A2F217FFF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SUST6_LIBSrest" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SUST6_LIBSrest!$A$1:$BI$24</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -3612,6 +3615,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BI24" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>